<commit_message>
feat: add 'send table' command to help menu and finalize bilingual mini-games UI
</commit_message>
<xml_diff>
--- a/מעקב תיקונים ושיפורים בוט.xlsx
+++ b/מעקב תיקונים ושיפורים בוט.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nirdahan/Documents/Projects/bet-joy-league-hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{001F71B5-9169-A846-B980-C6BCC1294877}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F5E3011-1D11-4842-A081-27C7A9895440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1060" yWindow="820" windowWidth="28100" windowHeight="17100" xr2:uid="{C6A91BF5-E6B2-464C-9FF8-1FB97885E412}"/>
+    <workbookView xWindow="5100" yWindow="940" windowWidth="28100" windowHeight="17100" xr2:uid="{C6A91BF5-E6B2-464C-9FF8-1FB97885E412}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>מס״ד</t>
   </si>
@@ -50,9 +50,6 @@
     <t>פיצ׳רים חדשים - טווח ארוך</t>
   </si>
   <si>
-    <t>תיקון מומחה ai</t>
-  </si>
-  <si>
     <t>הוספת אפשרות זוכה בטורניר</t>
   </si>
   <si>
@@ -77,9 +74,6 @@
     <t>הימור תוצאה מדויקת לא קשור לזהות המנצחת - אפשר לקבל ניקוד גם רק על זהות המנצחת</t>
   </si>
   <si>
-    <t>ליגה ציבורית - אי אפשר לחבר לווטסאפ</t>
-  </si>
-  <si>
     <t>לבדוק אם טופל</t>
   </si>
   <si>
@@ -92,28 +86,46 @@
     <t>בראקט למונדיאל</t>
   </si>
   <si>
-    <t>תיקון ״ניצח״ ל-״זכה ב-״</t>
-  </si>
-  <si>
     <t>לבדוק שיש מעלה לפרליי ושהוא באמת יודע לזהות שההימור בא ביחד</t>
   </si>
   <si>
-    <t>תיקון נוסחי הודעת ווטסאפ</t>
-  </si>
-  <si>
-    <t>הודעת אימות למשתמשים שחוברו</t>
-  </si>
-  <si>
-    <t>חיבור מנהלים</t>
-  </si>
-  <si>
-    <t>צפייה במספרי הטלפון במשתמשים בדאשבורד</t>
-  </si>
-  <si>
     <t>יציאה אוטומטית מקבוצות לא מקושרות</t>
   </si>
   <si>
-    <t>פקודות שאשפר לשלוח בקבוצות</t>
+    <t>תיאור אוטומטי לקבוצות שהבוט יוצר</t>
+  </si>
+  <si>
+    <t>תיקון מומחה ai - הסתרה שלו עד שעובד</t>
+  </si>
+  <si>
+    <t>חיבור מנהלים וריסטארטים</t>
+  </si>
+  <si>
+    <t>הודעות featured גם בווטסאפ</t>
+  </si>
+  <si>
+    <t>סגירת הימור 10 דקות לפני שריקת הפתיחה</t>
+  </si>
+  <si>
+    <t>תקלה ברישום רפרל וגוגל</t>
+  </si>
+  <si>
+    <t>תקלה בבחירת שם משתמש</t>
+  </si>
+  <si>
+    <t>הודעת סטטוס קבוצתית - ״טבלה״</t>
+  </si>
+  <si>
+    <t>תזמון שליחת טבלה מותאם אישית - באתר כולל תזכורת</t>
+  </si>
+  <si>
+    <t>בדיקת הודעות מתוזמנות - טבלה ומשחקים</t>
+  </si>
+  <si>
+    <t>תרגומים לאתגרים</t>
+  </si>
+  <si>
+    <t>ליגת טורניר - רק זהות מנצחת ותוצאות מדויקות (?)</t>
   </si>
 </sst>
 </file>
@@ -168,7 +180,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -191,11 +203,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -212,7 +235,13 @@
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -555,7 +584,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8549A035-1394-5E47-9754-56D43224C5A1}">
-  <dimension ref="A1:G29"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="49" bestFit="1" customWidth="1"/>
@@ -581,85 +610,87 @@
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>9</v>
+      <c r="B2" s="6" t="s">
+        <v>8</v>
       </c>
       <c r="C2" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="1" t="s">
         <v>4</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>15</v>
+      <c r="B3" s="6" t="s">
+        <v>13</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="C4" s="5" t="s">
+      <c r="B4" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="8" t="s">
         <v>12</v>
-      </c>
-      <c r="D4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" s="6" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>16</v>
+      <c r="B5" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>18</v>
+      <c r="B6" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="C6" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1" t="s">
-        <v>19</v>
+      <c r="B7" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>17</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
@@ -667,18 +698,20 @@
         <v>7</v>
       </c>
       <c r="B8" s="1"/>
-      <c r="C8" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="1"/>
+      <c r="C8" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>8</v>
       </c>
       <c r="B9" s="1"/>
-      <c r="C9" s="1" t="s">
-        <v>23</v>
+      <c r="C9" s="7" t="s">
+        <v>22</v>
       </c>
       <c r="D9" s="1"/>
     </row>
@@ -687,29 +720,37 @@
         <v>9</v>
       </c>
       <c r="B10" s="1"/>
-      <c r="C10" s="1" t="s">
-        <v>24</v>
+      <c r="C10" s="6" t="s">
+        <v>26</v>
       </c>
       <c r="D10" s="1"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="1"/>
+      <c r="A11" s="1">
+        <v>10</v>
+      </c>
       <c r="B11" s="1"/>
-      <c r="C11" s="1" t="s">
-        <v>25</v>
+      <c r="C11" s="6" t="s">
+        <v>28</v>
       </c>
       <c r="D11" s="1"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="1"/>
+    <row r="12" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="A12" s="1">
+        <v>11</v>
+      </c>
       <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
+      <c r="C12" s="5" t="s">
+        <v>11</v>
+      </c>
       <c r="D12" s="1"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
+      <c r="C13" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="D13" s="1"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
@@ -772,42 +813,6 @@
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="1"/>
-      <c r="B24" s="1"/>
-      <c r="C24" s="1"/>
-      <c r="D24" s="1"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="1"/>
-      <c r="B25" s="1"/>
-      <c r="C25" s="1"/>
-      <c r="D25" s="1"/>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A26" s="1"/>
-      <c r="B26" s="1"/>
-      <c r="C26" s="1"/>
-      <c r="D26" s="1"/>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A27" s="1"/>
-      <c r="B27" s="1"/>
-      <c r="C27" s="1"/>
-      <c r="D27" s="1"/>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A28" s="1"/>
-      <c r="B28" s="1"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A29" s="1"/>
-      <c r="B29" s="1"/>
-      <c r="C29" s="1"/>
-      <c r="D29" s="1"/>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: enforce 3-attempt limit for mini-games and update UI labels in challenges hub
</commit_message>
<xml_diff>
--- a/מעקב תיקונים ושיפורים בוט.xlsx
+++ b/מעקב תיקונים ושיפורים בוט.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nirdahan/Documents/Projects/bet-joy-league-hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F5E3011-1D11-4842-A081-27C7A9895440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25FDEBE7-C3D8-F348-86CD-795C4F1FBC84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5100" yWindow="940" windowWidth="28100" windowHeight="17100" xr2:uid="{C6A91BF5-E6B2-464C-9FF8-1FB97885E412}"/>
+    <workbookView xWindow="1060" yWindow="820" windowWidth="28100" windowHeight="17100" xr2:uid="{C6A91BF5-E6B2-464C-9FF8-1FB97885E412}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>מס״ד</t>
   </si>
@@ -56,9 +56,6 @@
     <t>הוספת הימור מותאם אישית</t>
   </si>
   <si>
-    <t>תיקון נראות אתר במחשב</t>
-  </si>
-  <si>
     <t>הימורים בזמן אמת</t>
   </si>
   <si>
@@ -89,9 +86,6 @@
     <t>לבדוק שיש מעלה לפרליי ושהוא באמת יודע לזהות שההימור בא ביחד</t>
   </si>
   <si>
-    <t>יציאה אוטומטית מקבוצות לא מקושרות</t>
-  </si>
-  <si>
     <t>תיאור אוטומטי לקבוצות שהבוט יוצר</t>
   </si>
   <si>
@@ -113,19 +107,40 @@
     <t>תקלה בבחירת שם משתמש</t>
   </si>
   <si>
-    <t>הודעת סטטוס קבוצתית - ״טבלה״</t>
-  </si>
-  <si>
-    <t>תזמון שליחת טבלה מותאם אישית - באתר כולל תזכורת</t>
-  </si>
-  <si>
-    <t>בדיקת הודעות מתוזמנות - טבלה ומשחקים</t>
-  </si>
-  <si>
     <t>תרגומים לאתגרים</t>
   </si>
   <si>
-    <t>ליגת טורניר - רק זהות מנצחת ותוצאות מדויקות (?)</t>
+    <t>תיקון מסך ברוכים הבאים ותוכן שעולה בו</t>
+  </si>
+  <si>
+    <t>משתמש שנמחק מופיע בלידר בורד</t>
+  </si>
+  <si>
+    <t>תיקון פרליי</t>
+  </si>
+  <si>
+    <t>הודעת ריסטארט ווטסאפ פעמיים</t>
+  </si>
+  <si>
+    <t>תקלה בתרגום קבוצות - ברנלי/בורנלי</t>
+  </si>
+  <si>
+    <t>שיפור הישגים</t>
+  </si>
+  <si>
+    <t xml:space="preserve">דוח מספר משתתפים </t>
+  </si>
+  <si>
+    <t>תזכורת לחבר ווטסאפ</t>
+  </si>
+  <si>
+    <t>שינוי ניקוד משחקים</t>
+  </si>
+  <si>
+    <t>חיבור כמה ליגות לקבוצה אחת</t>
+  </si>
+  <si>
+    <t>תקלה בסיכויי ווטסאפ</t>
   </si>
 </sst>
 </file>
@@ -148,7 +163,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -176,6 +191,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -218,7 +245,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -232,17 +259,20 @@
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -611,10 +641,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>8</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>19</v>
+        <v>7</v>
+      </c>
+      <c r="C2" s="9" t="s">
+        <v>30</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>4</v>
@@ -625,10 +655,10 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>6</v>
+        <v>12</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>25</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>5</v>
@@ -639,16 +669,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>20</v>
-      </c>
-      <c r="C4" s="1" t="s">
         <v>18</v>
       </c>
+      <c r="C4" s="6" t="s">
+        <v>26</v>
+      </c>
       <c r="D4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>12</v>
+        <v>6</v>
+      </c>
+      <c r="G4" s="5" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
@@ -656,13 +686,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
@@ -670,13 +700,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
@@ -687,133 +717,166 @@
         <v>27</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" s="1"/>
-      <c r="C8" s="6" t="s">
-        <v>21</v>
+      <c r="B8" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>20</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" s="1"/>
-      <c r="C9" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="1"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B9" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="34" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="D10" s="1"/>
+      <c r="B10" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="B11" s="1"/>
-      <c r="C11" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="1"/>
-    </row>
-    <row r="12" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+      <c r="B11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>11</v>
       </c>
       <c r="B12" s="1"/>
-      <c r="C12" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D12" s="1"/>
+      <c r="C12" s="1"/>
+      <c r="D12" s="1" t="s">
+        <v>33</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="1"/>
+      <c r="A13" s="1">
+        <v>12</v>
+      </c>
       <c r="B13" s="1"/>
-      <c r="C13" s="1" t="s">
-        <v>29</v>
-      </c>
+      <c r="C13" s="1"/>
       <c r="D13" s="1"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="1"/>
+      <c r="A14" s="1">
+        <v>13</v>
+      </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="1"/>
+      <c r="A15" s="1">
+        <v>14</v>
+      </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="1"/>
+      <c r="A16" s="1">
+        <v>15</v>
+      </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
+      <c r="A17" s="1">
+        <v>16</v>
+      </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="1"/>
+      <c r="A18" s="1">
+        <v>17</v>
+      </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="1"/>
+      <c r="A19" s="1">
+        <v>18</v>
+      </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="1"/>
+      <c r="A20" s="1">
+        <v>19</v>
+      </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="1"/>
+      <c r="A21" s="1">
+        <v>20</v>
+      </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A22" s="1"/>
+      <c r="A22" s="1">
+        <v>21</v>
+      </c>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="1"/>
+      <c r="A23" s="1">
+        <v>22</v>
+      </c>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Fix syntax errors, missing API imports, and TypeScript overload issues in useApi and AdminDashboard
</commit_message>
<xml_diff>
--- a/מעקב תיקונים ושיפורים בוט.xlsx
+++ b/מעקב תיקונים ושיפורים בוט.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nirdahan/Documents/Projects/bet-joy-league-hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25FDEBE7-C3D8-F348-86CD-795C4F1FBC84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54D76AAB-07C3-9543-AFBA-E0E4CBEB5936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1060" yWindow="820" windowWidth="28100" windowHeight="17100" xr2:uid="{C6A91BF5-E6B2-464C-9FF8-1FB97885E412}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{C6A91BF5-E6B2-464C-9FF8-1FB97885E412}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>מס״ד</t>
   </si>
@@ -59,9 +59,6 @@
     <t>הימורים בזמן אמת</t>
   </si>
   <si>
-    <t>חיבור בוט ווטסאפ</t>
-  </si>
-  <si>
     <t>שיווק האתר</t>
   </si>
   <si>
@@ -71,9 +68,6 @@
     <t>הימור תוצאה מדויקת לא קשור לזהות המנצחת - אפשר לקבל ניקוד גם רק על זהות המנצחת</t>
   </si>
   <si>
-    <t>לבדוק אם טופל</t>
-  </si>
-  <si>
     <t>משחקים שלא עובדו - יצירת מנגנון שמוודא שלא פספסנו אף משחק פעם ביום</t>
   </si>
   <si>
@@ -104,24 +98,15 @@
     <t>תקלה ברישום רפרל וגוגל</t>
   </si>
   <si>
-    <t>תקלה בבחירת שם משתמש</t>
-  </si>
-  <si>
     <t>תרגומים לאתגרים</t>
   </si>
   <si>
-    <t>תיקון מסך ברוכים הבאים ותוכן שעולה בו</t>
-  </si>
-  <si>
     <t>משתמש שנמחק מופיע בלידר בורד</t>
   </si>
   <si>
     <t>תיקון פרליי</t>
   </si>
   <si>
-    <t>הודעת ריסטארט ווטסאפ פעמיים</t>
-  </si>
-  <si>
     <t>תקלה בתרגום קבוצות - ברנלי/בורנלי</t>
   </si>
   <si>
@@ -131,16 +116,19 @@
     <t xml:space="preserve">דוח מספר משתתפים </t>
   </si>
   <si>
-    <t>תזכורת לחבר ווטסאפ</t>
-  </si>
-  <si>
-    <t>שינוי ניקוד משחקים</t>
-  </si>
-  <si>
     <t>חיבור כמה ליגות לקבוצה אחת</t>
   </si>
   <si>
     <t>תקלה בסיכויי ווטסאפ</t>
+  </si>
+  <si>
+    <t>תוקן - לבדוק שעובד</t>
+  </si>
+  <si>
+    <t>תמיכה מלאה בעברית ובאנגלית</t>
+  </si>
+  <si>
+    <t>שינוי סיסמא</t>
   </si>
 </sst>
 </file>
@@ -163,7 +151,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -179,12 +167,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF74F"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -245,7 +227,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -256,22 +238,13 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -614,266 +587,280 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8549A035-1394-5E47-9754-56D43224C5A1}">
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="49" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="30.5703125" customWidth="1"/>
+    <col min="3" max="3" width="57.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="30.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>1</v>
       </c>
-      <c r="B2" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="9" t="s">
-        <v>30</v>
-      </c>
-      <c r="D2" s="1" t="s">
+      <c r="B2" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="6" t="s">
-        <v>12</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>25</v>
+      <c r="B3" s="1"/>
+      <c r="C3" s="1" t="s">
+        <v>22</v>
       </c>
       <c r="D3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>3</v>
       </c>
-      <c r="B4" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>26</v>
+      <c r="B4" s="1"/>
+      <c r="C4" s="1" t="s">
+        <v>13</v>
       </c>
       <c r="D4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="G4" s="5" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>15</v>
+      <c r="B5" s="1"/>
+      <c r="C5" s="1" t="s">
+        <v>16</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+        <v>30</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B6" s="1"/>
+      <c r="C6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B7" s="1"/>
+      <c r="C7" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" s="6" t="s">
-        <v>28</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="B8" s="1"/>
+      <c r="C8" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" s="1"/>
+      <c r="E8" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" s="6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" s="6" t="s">
+      <c r="B9" s="1"/>
+      <c r="C9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="1"/>
+      <c r="E9" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="34" x14ac:dyDescent="0.2">
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" s="6" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" s="8" t="s">
+      <c r="B10" s="1"/>
+      <c r="C10" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D10" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D10" s="1"/>
+      <c r="E10" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>34</v>
-      </c>
+      <c r="B11" s="1"/>
       <c r="C11" s="1"/>
-      <c r="D11" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D11" s="1"/>
+      <c r="E11" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>11</v>
       </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
-      <c r="D12" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D12" s="1"/>
+      <c r="E12" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>12</v>
       </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E13" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>13</v>
       </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>14</v>
       </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="E15" s="1"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>15</v>
       </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>16</v>
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E17" s="1"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>17</v>
       </c>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>18</v>
       </c>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E19" s="1"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>19</v>
       </c>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>20</v>
       </c>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E21" s="1"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>21</v>
       </c>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="E22" s="1"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>22</v>
       </c>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
+      <c r="E23" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
UI: Minor adjustments and code cleanup.
</commit_message>
<xml_diff>
--- a/מעקב תיקונים ושיפורים בוט.xlsx
+++ b/מעקב תיקונים ושיפורים בוט.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nirdahan/Documents/Projects/bet-joy-league-hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54D76AAB-07C3-9543-AFBA-E0E4CBEB5936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A89FD12-E212-C34E-9450-3CC260DF8B21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{C6A91BF5-E6B2-464C-9FF8-1FB97885E412}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>מס״ד</t>
   </si>
@@ -129,6 +129,9 @@
   </si>
   <si>
     <t>שינוי סיסמא</t>
+  </si>
+  <si>
+    <t>שינוי מסך פתיחה - הוספת מצב אורח</t>
   </si>
 </sst>
 </file>
@@ -227,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -245,6 +248,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -623,9 +629,7 @@
       <c r="C2" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D2" s="6" t="s">
-        <v>25</v>
-      </c>
+      <c r="D2" s="7"/>
       <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
@@ -638,9 +642,7 @@
       <c r="C3" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="D3" s="1"/>
       <c r="E3" s="1" t="s">
         <v>5</v>
       </c>
@@ -653,9 +655,7 @@
       <c r="C4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="D4" s="1" t="s">
-        <v>20</v>
-      </c>
+      <c r="D4" s="1"/>
       <c r="E4" s="1" t="s">
         <v>6</v>
       </c>
@@ -668,9 +668,7 @@
       <c r="C5" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="1" t="s">
-        <v>30</v>
-      </c>
+      <c r="D5" s="1"/>
       <c r="E5" s="1" t="s">
         <v>7</v>
       </c>
@@ -683,6 +681,7 @@
       <c r="C6" s="1" t="s">
         <v>17</v>
       </c>
+      <c r="D6" s="1"/>
       <c r="E6" s="1" t="s">
         <v>8</v>
       </c>
@@ -710,7 +709,7 @@
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1" t="s">
-        <v>11</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -744,7 +743,9 @@
         <v>10</v>
       </c>
       <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
+      <c r="C11" s="1" t="s">
+        <v>27</v>
+      </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1" t="s">
         <v>14</v>
@@ -755,7 +756,9 @@
         <v>11</v>
       </c>
       <c r="B12" s="1"/>
-      <c r="C12" s="1"/>
+      <c r="C12" s="1" t="s">
+        <v>11</v>
+      </c>
       <c r="D12" s="1"/>
       <c r="E12" s="1" t="s">
         <v>26</v>
@@ -766,7 +769,9 @@
         <v>12</v>
       </c>
       <c r="B13" s="1"/>
-      <c r="C13" s="1"/>
+      <c r="C13" s="1" t="s">
+        <v>30</v>
+      </c>
       <c r="D13" s="1"/>
       <c r="E13" s="1" t="s">
         <v>29</v>
@@ -777,9 +782,13 @@
         <v>13</v>
       </c>
       <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
+      <c r="C14" s="7" t="s">
+        <v>31</v>
+      </c>
       <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
+      <c r="E14" s="6" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A15" s="1">

</xml_diff>

<commit_message>
feat: restrict game visibility and improve system performance
</commit_message>
<xml_diff>
--- a/מעקב תיקונים ושיפורים בוט.xlsx
+++ b/מעקב תיקונים ושיפורים בוט.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nirdahan/Documents/Projects/bet-joy-league-hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0A89FD12-E212-C34E-9450-3CC260DF8B21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4291301-852E-0448-BA3F-F3E70192CCD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{C6A91BF5-E6B2-464C-9FF8-1FB97885E412}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17360" xr2:uid="{C6A91BF5-E6B2-464C-9FF8-1FB97885E412}"/>
   </bookViews>
   <sheets>
     <sheet name="גיליון1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>מס״ד</t>
   </si>
@@ -65,15 +65,9 @@
     <t>קניית נקודות</t>
   </si>
   <si>
-    <t>הימור תוצאה מדויקת לא קשור לזהות המנצחת - אפשר לקבל ניקוד גם רק על זהות המנצחת</t>
-  </si>
-  <si>
     <t>משחקים שלא עובדו - יצירת מנגנון שמוודא שלא פספסנו אף משחק פעם ביום</t>
   </si>
   <si>
-    <t>פנייה למנהלים</t>
-  </si>
-  <si>
     <t>בראקט למונדיאל</t>
   </si>
   <si>
@@ -89,9 +83,6 @@
     <t>חיבור מנהלים וריסטארטים</t>
   </si>
   <si>
-    <t>הודעות featured גם בווטסאפ</t>
-  </si>
-  <si>
     <t>סגירת הימור 10 דקות לפני שריקת הפתיחה</t>
   </si>
   <si>
@@ -131,7 +122,10 @@
     <t>שינוי סיסמא</t>
   </si>
   <si>
-    <t>שינוי מסך פתיחה - הוספת מצב אורח</t>
+    <t>התראות בווטסאפ מותאמות אישית</t>
+  </si>
+  <si>
+    <t>משתמש מחוק מופיע ברישומים</t>
   </si>
 </sst>
 </file>
@@ -250,7 +244,7 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -610,7 +604,7 @@
         <v>1</v>
       </c>
       <c r="C1" s="5" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D1" s="3" t="s">
         <v>2</v>
@@ -624,12 +618,14 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" s="7"/>
+        <v>18</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>28</v>
+      </c>
       <c r="E2" s="1" t="s">
         <v>4</v>
       </c>
@@ -638,9 +634,11 @@
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="1"/>
+      <c r="B3" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="C3" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D3" s="1"/>
       <c r="E3" s="1" t="s">
@@ -653,7 +651,7 @@
       </c>
       <c r="B4" s="1"/>
       <c r="C4" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D4" s="1"/>
       <c r="E4" s="1" t="s">
@@ -666,7 +664,7 @@
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D5" s="1"/>
       <c r="E5" s="1" t="s">
@@ -679,7 +677,7 @@
       </c>
       <c r="B6" s="1"/>
       <c r="C6" s="1" t="s">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="D6" s="1"/>
       <c r="E6" s="1" t="s">
@@ -692,11 +690,11 @@
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="D7" s="1"/>
       <c r="E7" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
@@ -705,11 +703,11 @@
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
@@ -718,11 +716,11 @@
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1" t="s">
-        <v>9</v>
+        <v>24</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -731,11 +729,11 @@
       </c>
       <c r="B10" s="1"/>
       <c r="C10" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
@@ -743,12 +741,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="1"/>
-      <c r="C11" s="1" t="s">
-        <v>27</v>
-      </c>
+      <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
@@ -756,12 +752,10 @@
         <v>11</v>
       </c>
       <c r="B12" s="1"/>
-      <c r="C12" s="1" t="s">
-        <v>11</v>
-      </c>
+      <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -769,12 +763,10 @@
         <v>12</v>
       </c>
       <c r="B13" s="1"/>
-      <c r="C13" s="1" t="s">
-        <v>30</v>
-      </c>
+      <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
@@ -782,12 +774,10 @@
         <v>13</v>
       </c>
       <c r="B14" s="1"/>
-      <c r="C14" s="7" t="s">
-        <v>31</v>
-      </c>
+      <c r="C14" s="7"/>
       <c r="D14" s="1"/>
       <c r="E14" s="6" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
feat: add bulk cleanup for anonymized users in admin dashboard
</commit_message>
<xml_diff>
--- a/מעקב תיקונים ושיפורים בוט.xlsx
+++ b/מעקב תיקונים ושיפורים בוט.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nirdahan/Documents/Projects/bet-joy-league-hub/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A4291301-852E-0448-BA3F-F3E70192CCD6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35CE83E3-0BA7-6441-A7F9-2C6188F1F4C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17360" xr2:uid="{C6A91BF5-E6B2-464C-9FF8-1FB97885E412}"/>
   </bookViews>
@@ -125,7 +125,7 @@
     <t>התראות בווטסאפ מותאמות אישית</t>
   </si>
   <si>
-    <t>משתמש מחוק מופיע ברישומים</t>
+    <t>תזכורת למי שלא הימר</t>
   </si>
 </sst>
 </file>
@@ -634,13 +634,13 @@
       <c r="A3" s="1">
         <v>2</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>29</v>
-      </c>
+      <c r="B3" s="1"/>
       <c r="C3" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="D3" s="1"/>
+      <c r="D3" s="1" t="s">
+        <v>29</v>
+      </c>
       <c r="E3" s="1" t="s">
         <v>5</v>
       </c>

</xml_diff>